<commit_message>
Regenerate analysis report and tables from full dataset
The committed report was stale, reporting $111,998.90 in sales across a
single region and category. Regenerated against the full cleaned dataset:
$14,915,600.82 across 8 regions, 3 categories and 5,496 orders.
</commit_message>
<xml_diff>
--- a/output/reports/analysis_tables.xlsx
+++ b/output/reports/analysis_tables.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="sales_by_region" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="sales_by_product_category" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="top_10_products_by_sales" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="profit_by_customer_segment" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="sales_by_order_priority" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="monthly_sales_trend" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="profit_by_product_category" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sales_by_region" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sales_by_product_category" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="top_10_products_by_sales" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="profit_by_customer_segment" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sales_by_order_priority" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="monthly_sales_trend" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="profit_by_product_category" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>